<commit_message>
Adjusted character orientation code
</commit_message>
<xml_diff>
--- a/Noir Wingman/Assets/Sheets/SamDiggumsIntro1.xlsx
+++ b/Noir Wingman/Assets/Sheets/SamDiggumsIntro1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\coles\OneDrive\Desktop\Noir Wingman\Assets\Sheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\coles\OneDrive\Desktop\NoirWingman\Noir Wingman\Assets\Sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F9BF4C6-FA0F-41DF-A135-1B041EB85BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD509611-B347-4536-8254-4547B7403B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" xr2:uid="{8ACFDE19-706B-4AD7-A091-DD6B157D164D}"/>
   </bookViews>
@@ -86,9 +86,6 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>*It wasn’t a bad night, but there was something off in the air- the kind of feeling that makes you check your back a little more than you normally would. Not that it’d do you any good. The day’s rain had melted in the late summer heat into a fog so thick you couldn’t see a muzzle flash from more than 10 feet away. |*The bar was nothing special. The lights flickered dimly, the bartender glowered from the corner, and it stank of cheap smokes and cheaper booze. You know the type. But, what was special- or at least, unusual- was the people drinking here on this strange, foggy evening. |Evening, Jules. |*Lieutenant Sam Diggums- as loyal as a blind mutt, and about as scary. My ex-partner on the force.|Hey, Sam. You've been drinking.|Hic- Yeah, only a little- Hic.|*He hasn’t been taking my resignation well. |Say, have ya found those files on the Baron’s disappearance for me?|What? Uh, no- sorry, I’ve been- uh- busy. Hic.|*Poor sap- he’s been drowning himself in drink. If I want him to get me those leads, I gotta find a way to sober him up- for good.|Look, buddy, you want some help? I’m not big on this whole, uh, romance thing, but I know people- it’s my job |Wouldja??? That’d- hic- mean a whole lot.|Yeah, least I could do.|*Now, let’s take a look at our suspe- I mean, candidates.</t>
-  </si>
-  <si>
     <t>Neutral|Angry|Neutral|Angry|Neutral|Sad|Sad|Neutral|Angry|Sad|Neutral|Sad|Happy|Angry</t>
   </si>
   <si>
@@ -99,19 +96,28 @@
   </si>
   <si>
     <t>0|0|3|0|1|3|0|1|3|0|1|2|1|0</t>
+  </si>
+  <si>
+    <t>*It wasn't a bad night, but there was something off in the air- the kind of feeling that makes you check your back a little more than you normally would. Not that it'd do you any good. The day's rain had melted in the late summer heat into a fog so thick you couldn't see a muzzle flash from more than 10 feet away. |*The bar was nothing special. The lights flickered dimly, the bartender glowered from the corner, and it stank of cheap smokes and cheaper booze. You know the type. But, what was special- or at least, unusual- was the people drinking here on this strange, foggy evening. |Evening, Jules. |*Lieutenant Sam Diggums- as loyal as a blind mutt, and about as scary. My ex-partner on the force.|Hey, Sam. You've been drinking.|Hic- Yeah, only a little- Hic.|*He hasn't been taking my resignation well. |Say, have ya found those files on the Baron's disappearance for me?|What? Uh, no- sorry, I've been- uh- busy. Hic.|*Poor sap- he's been drowning himself in drink. If I want him to get me those leads, I gotta find a way to sober him up- for good.|Look, buddy, you want some help? I'm not big on this whole, uh, romance thing, but I know people- it's my job |Wouldja??? That'd- hic- mean a whole lot.|Yeah, least I could do.|*Now, let's take a look at our suspe- I mean, candidates.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -134,9 +140,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -532,42 +541,42 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="174" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" ht="182.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>14</v>
       </c>
       <c r="B2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" t="s">
-        <v>18</v>
-      </c>
       <c r="F2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M2">
         <v>0</v>

</xml_diff>